<commit_message>
Update UI/UX branding to CCL Offshore Roster AI and refresh labels
</commit_message>
<xml_diff>
--- a/offshore roaster/April - July schedule.xlsx
+++ b/offshore roaster/April - July schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CCL-04\ai_project\offshore roaster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D5E207-A027-4FDC-BB0F-114CA43B38A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B56E4552-0167-4B46-965F-25B5D3379BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{114A9C9E-D32A-4C11-8C68-A41F13B01295}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="89">
   <si>
     <t>Date</t>
   </si>
@@ -167,12 +166,6 @@
   </si>
   <si>
     <t>Week 11</t>
-  </si>
-  <si>
-    <t>Week 12</t>
-  </si>
-  <si>
-    <t>Week 13</t>
   </si>
   <si>
     <t>Rohit 7AM - 1PM</t>
@@ -461,6 +454,18 @@
   </si>
   <si>
     <t>Vasu</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Suraj/Akhil</t>
+  </si>
+  <si>
+    <t>Siva (1 10 PM)/Gopi(3PM to 12AM)</t>
+  </si>
+  <si>
+    <t>Akhil/Gopi</t>
   </si>
 </sst>
 </file>
@@ -550,7 +555,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -610,25 +615,75 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -642,6 +697,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -976,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6035BA0-F57A-4AAC-9051-A855D20937A2}">
-  <dimension ref="A1:G151"/>
+  <dimension ref="A1:H235"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.6640625" customWidth="1"/>
@@ -994,13 +1072,13 @@
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="7" t="s">
@@ -1013,31 +1091,31 @@
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
@@ -1050,7 +1128,7 @@
         <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>16</v>
@@ -1071,7 +1149,7 @@
         <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>16</v>
@@ -1092,7 +1170,7 @@
         <v>13</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>18</v>
@@ -1115,7 +1193,7 @@
         <v>13</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>18</v>
@@ -1138,10 +1216,10 @@
         <v>13</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>14</v>
@@ -1156,13 +1234,13 @@
         <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>28</v>
@@ -1179,13 +1257,13 @@
         <v>12</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="E11" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>28</v>
@@ -1207,7 +1285,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1218,7 +1296,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1229,7 +1307,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -1239,15 +1317,15 @@
       <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
@@ -1402,7 +1480,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1421,15 +1499,15 @@
       <c r="G25" s="3"/>
     </row>
     <row r="26" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
@@ -1584,7 +1662,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1603,15 +1681,15 @@
       <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
@@ -1766,7 +1844,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1776,15 +1854,15 @@
       <c r="G44" s="3"/>
     </row>
     <row r="45" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
@@ -1890,7 +1968,7 @@
         <v>14</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
@@ -1941,10 +2019,10 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -1953,15 +2031,15 @@
       <c r="G53" s="3"/>
     </row>
     <row r="54" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A54" s="9" t="s">
+      <c r="A54" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B54" s="9"/>
-      <c r="C54" s="9"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="9"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
@@ -1970,13 +2048,13 @@
       <c r="B55" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C55" s="8" t="s">
+      <c r="C55" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D55" s="8" t="s">
+      <c r="D55" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E55" s="8" t="s">
+      <c r="E55" s="6" t="s">
         <v>3</v>
       </c>
       <c r="F55" s="7" t="s">
@@ -1989,9 +2067,9 @@
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="7"/>
       <c r="B56" s="7"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="8"/>
-      <c r="E56" s="8"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6"/>
       <c r="F56" s="7"/>
       <c r="G56" s="7"/>
     </row>
@@ -2036,7 +2114,7 @@
         <v>22</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
@@ -2092,16 +2170,16 @@
         <v>14</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="18" x14ac:dyDescent="0.35">
@@ -2115,21 +2193,21 @@
         <v>14</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -2140,7 +2218,7 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -2159,15 +2237,15 @@
       <c r="G65" s="3"/>
     </row>
     <row r="66" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A66" s="10" t="s">
+      <c r="A66" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B66" s="11"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="11"/>
-      <c r="G66" s="12"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="10"/>
+      <c r="E66" s="10"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="11"/>
     </row>
     <row r="67" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
@@ -2180,7 +2258,7 @@
         <v>14</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>16</v>
@@ -2189,7 +2267,7 @@
         <v>17</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="18" x14ac:dyDescent="0.35">
@@ -2203,7 +2281,7 @@
         <v>14</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>16</v>
@@ -2212,7 +2290,7 @@
         <v>17</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
@@ -2226,14 +2304,14 @@
         <v>14</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
@@ -2247,14 +2325,14 @@
         <v>14</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
@@ -2268,14 +2346,14 @@
         <v>14</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
@@ -2289,7 +2367,7 @@
         <v>14</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E72" s="3" t="s">
         <v>19</v>
@@ -2298,7 +2376,7 @@
         <v>31</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
@@ -2312,7 +2390,7 @@
         <v>14</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>19</v>
@@ -2321,12 +2399,12 @@
         <v>31</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -2336,15 +2414,15 @@
       <c r="G74" s="3"/>
     </row>
     <row r="75" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A75" s="10" t="s">
+      <c r="A75" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B75" s="11"/>
-      <c r="C75" s="11"/>
-      <c r="D75" s="11"/>
-      <c r="E75" s="11"/>
-      <c r="F75" s="11"/>
-      <c r="G75" s="12"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="10"/>
+      <c r="F75" s="10"/>
+      <c r="G75" s="11"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
@@ -2387,7 +2465,7 @@
         <v>13</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
@@ -2501,7 +2579,7 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -2511,15 +2589,15 @@
       <c r="G83" s="3"/>
     </row>
     <row r="84" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A84" s="9" t="s">
+      <c r="A84" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B84" s="9"/>
-      <c r="C84" s="9"/>
-      <c r="D84" s="9"/>
-      <c r="E84" s="9"/>
-      <c r="F84" s="9"/>
-      <c r="G84" s="9"/>
+      <c r="B84" s="8"/>
+      <c r="C84" s="8"/>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="8"/>
+      <c r="G84" s="8"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
@@ -2595,16 +2673,16 @@
         <v>13</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
@@ -2618,16 +2696,16 @@
         <v>13</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
@@ -2650,7 +2728,7 @@
         <v>31</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
@@ -2673,12 +2751,12 @@
         <v>31</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -2688,15 +2766,15 @@
       <c r="G92" s="3"/>
     </row>
     <row r="93" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A93" s="9" t="s">
+      <c r="A93" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B93" s="9"/>
-      <c r="C93" s="9"/>
-      <c r="D93" s="9"/>
-      <c r="E93" s="9"/>
-      <c r="F93" s="9"/>
-      <c r="G93" s="9"/>
+      <c r="B93" s="8"/>
+      <c r="C93" s="8"/>
+      <c r="D93" s="8"/>
+      <c r="E93" s="8"/>
+      <c r="F93" s="8"/>
+      <c r="G93" s="8"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
@@ -2706,7 +2784,7 @@
         <v>6</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>21</v>
@@ -2718,7 +2796,7 @@
         <v>13</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
@@ -2729,7 +2807,7 @@
         <v>7</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>21</v>
@@ -2741,7 +2819,7 @@
         <v>13</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
@@ -2773,7 +2851,7 @@
         <v>9</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>21</v>
@@ -2855,7 +2933,7 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -2865,15 +2943,15 @@
       <c r="G101" s="3"/>
     </row>
     <row r="102" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A102" s="9" t="s">
+      <c r="A102" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B102" s="9"/>
-      <c r="C102" s="9"/>
-      <c r="D102" s="9"/>
-      <c r="E102" s="9"/>
-      <c r="F102" s="9"/>
-      <c r="G102" s="9"/>
+      <c r="B102" s="8"/>
+      <c r="C102" s="8"/>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="8"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
@@ -3028,7 +3106,7 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -3038,15 +3116,15 @@
       <c r="G110" s="3"/>
     </row>
     <row r="111" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A111" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B111" s="9"/>
-      <c r="C111" s="9"/>
-      <c r="D111" s="9"/>
-      <c r="E111" s="9"/>
-      <c r="F111" s="9"/>
-      <c r="G111" s="9"/>
+      <c r="A111" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B111" s="8"/>
+      <c r="C111" s="8"/>
+      <c r="D111" s="8"/>
+      <c r="E111" s="8"/>
+      <c r="F111" s="8"/>
+      <c r="G111" s="8"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
@@ -3201,7 +3279,7 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -3211,15 +3289,15 @@
       <c r="G119" s="3"/>
     </row>
     <row r="120" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A120" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B120" s="9"/>
-      <c r="C120" s="9"/>
-      <c r="D120" s="9"/>
-      <c r="E120" s="9"/>
-      <c r="F120" s="9"/>
-      <c r="G120" s="9"/>
+      <c r="A120" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B120" s="8"/>
+      <c r="C120" s="8"/>
+      <c r="D120" s="8"/>
+      <c r="E120" s="8"/>
+      <c r="F120" s="8"/>
+      <c r="G120" s="8"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
@@ -3374,80 +3452,2038 @@
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A129" s="1"/>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A130" s="1"/>
-    </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A131" s="1"/>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A132" s="1"/>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A133" s="1"/>
-    </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A134" s="1"/>
-    </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A135" s="1"/>
-    </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A136" s="1"/>
-    </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A137" s="1"/>
-    </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A138" s="1"/>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A139" s="1"/>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A140" s="1"/>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A141" s="1"/>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A142" s="1"/>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A143" s="1"/>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A144" s="1"/>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A145" s="1"/>
-    </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A146" s="1"/>
-    </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A147" s="1"/>
-    </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A148" s="1"/>
-    </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A149" s="1"/>
-    </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A150" s="1"/>
-    </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A151" s="1"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="A129" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B129" s="13"/>
+      <c r="C129" s="13"/>
+      <c r="D129" s="13"/>
+      <c r="E129" s="13"/>
+      <c r="F129" s="13"/>
+      <c r="G129" s="13"/>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A130" s="2">
+        <v>46216</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G130" s="3"/>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A131" s="2">
+        <v>46217</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E131" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G131" s="3"/>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A132" s="2">
+        <v>46218</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G132" s="3"/>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A133" s="2">
+        <v>46219</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G133" s="3"/>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A134" s="2">
+        <v>46220</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G134" s="3"/>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A135" s="2">
+        <v>46221</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E135" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G135" s="3"/>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A136" s="2">
+        <v>46222</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G136" s="3"/>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A137" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G137" s="14"/>
+    </row>
+    <row r="138" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="A138" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B138" s="13"/>
+      <c r="C138" s="13"/>
+      <c r="D138" s="13"/>
+      <c r="E138" s="13"/>
+      <c r="F138" s="13"/>
+      <c r="G138" s="13"/>
+      <c r="H138" s="15"/>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A139" s="2">
+        <v>46223</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E139" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G139" s="3"/>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A140" s="2">
+        <v>46224</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G140" s="3"/>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A141" s="2">
+        <v>46225</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E141" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F141" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G141" s="3"/>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A142" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G142" s="3"/>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A143" s="2">
+        <v>46227</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E143" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G143" s="3"/>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A144" s="2">
+        <v>46228</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G144" s="3"/>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A145" s="2">
+        <v>46229</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E145" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G145" s="3"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A146" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G146" s="14"/>
+    </row>
+    <row r="147" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A147" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B147" s="16"/>
+      <c r="C147" s="16"/>
+      <c r="D147" s="16"/>
+      <c r="E147" s="16"/>
+      <c r="F147" s="16"/>
+      <c r="G147" s="17"/>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A148" s="2">
+        <v>46230</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G148" s="3"/>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A149" s="2">
+        <v>46231</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E149" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F149" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G149" s="3"/>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A150" s="2">
+        <v>46232</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E150" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G150" s="3"/>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A151" s="2">
+        <v>46233</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E151" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F151" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G151" s="3"/>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A152" s="2">
+        <v>46234</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E152" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G152" s="3"/>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A153" s="2">
+        <v>46235</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C153" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D153" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E153" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F153" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G153" s="3"/>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A154" s="2">
+        <v>46236</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E154" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G154" s="3"/>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A156" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B156" s="18"/>
+      <c r="C156" s="18"/>
+      <c r="D156" s="18"/>
+      <c r="E156" s="18"/>
+      <c r="F156" s="18"/>
+      <c r="G156" s="18"/>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A157" s="22">
+        <v>46237</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D157" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E157" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F157" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G157" s="3"/>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A158" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D158" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E158" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G158" s="3"/>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A159" s="1">
+        <v>46239</v>
+      </c>
+      <c r="B159" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D159" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E159" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F159" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G159" s="3"/>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A160" s="1">
+        <v>46240</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E160" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F160" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G160" s="3"/>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A161" s="1">
+        <v>46241</v>
+      </c>
+      <c r="B161" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C161" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D161" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E161" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F161" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G161" s="3"/>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A162" s="1">
+        <v>46242</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E162" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G162" s="3"/>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A163" s="1">
+        <v>46243</v>
+      </c>
+      <c r="B163" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C163" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D163" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E163" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F163" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G163" s="19"/>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A164" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B164" s="3"/>
+      <c r="C164" s="3"/>
+      <c r="D164" s="3"/>
+      <c r="E164" s="3"/>
+      <c r="F164" s="3"/>
+      <c r="G164" s="3"/>
+    </row>
+    <row r="165" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A165" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B165" s="8"/>
+      <c r="C165" s="8"/>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8"/>
+      <c r="F165" s="8"/>
+      <c r="G165" s="8"/>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A166" s="2">
+        <v>46244</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D166" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E166" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F166" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G166" s="3"/>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A167" s="2">
+        <v>46245</v>
+      </c>
+      <c r="B167" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C167" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D167" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E167" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F167" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G167" s="3"/>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A168" s="2">
+        <v>46246</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C168" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E168" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F168" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G168" s="3"/>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A169" s="2">
+        <v>46247</v>
+      </c>
+      <c r="B169" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C169" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D169" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E169" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F169" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G169" s="3"/>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A170" s="2">
+        <v>46248</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C170" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D170" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E170" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F170" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G170" s="3"/>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A171" s="2">
+        <v>46249</v>
+      </c>
+      <c r="B171" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C171" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D171" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E171" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F171" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G171" s="3"/>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A172" s="2">
+        <v>46250</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C172" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D172" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E172" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F172" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G172" s="3"/>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A173" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B173" s="3"/>
+      <c r="C173" s="3"/>
+      <c r="D173" s="3"/>
+      <c r="E173" s="3"/>
+      <c r="F173" s="3"/>
+      <c r="G173" s="3"/>
+    </row>
+    <row r="174" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A174" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B174" s="20"/>
+      <c r="C174" s="20"/>
+      <c r="D174" s="20"/>
+      <c r="E174" s="20"/>
+      <c r="F174" s="20"/>
+      <c r="G174" s="20"/>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A175" s="2">
+        <v>46251</v>
+      </c>
+      <c r="B175" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C175" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D175" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E175" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F175" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G175" s="3"/>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A176" s="2">
+        <v>46252</v>
+      </c>
+      <c r="B176" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C176" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D176" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E176" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F176" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G176" s="3"/>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A177" s="2">
+        <v>46253</v>
+      </c>
+      <c r="B177" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D177" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E177" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F177" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G177" s="3"/>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A178" s="2">
+        <v>46254</v>
+      </c>
+      <c r="B178" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D178" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E178" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F178" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G178" s="3"/>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A179" s="2">
+        <v>46255</v>
+      </c>
+      <c r="B179" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D179" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E179" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F179" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G179" s="3"/>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A180" s="2">
+        <v>46256</v>
+      </c>
+      <c r="B180" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D180" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E180" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F180" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G180" s="3"/>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A181" s="2">
+        <v>46257</v>
+      </c>
+      <c r="B181" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C181" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D181" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E181" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F181" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G181" s="3"/>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A182" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B182" s="21"/>
+      <c r="C182" s="3"/>
+      <c r="D182" s="3"/>
+      <c r="E182" s="3"/>
+      <c r="F182" s="3"/>
+      <c r="G182" s="3"/>
+    </row>
+    <row r="183" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A183" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B183" s="20"/>
+      <c r="C183" s="20"/>
+      <c r="D183" s="20"/>
+      <c r="E183" s="20"/>
+      <c r="F183" s="20"/>
+      <c r="G183" s="20"/>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A184" s="2">
+        <v>46258</v>
+      </c>
+      <c r="B184" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D184" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E184" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F184" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G184" s="3"/>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A185" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B185" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C185" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D185" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E185" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F185" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G185" s="3"/>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A186" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B186" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C186" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D186" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E186" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F186" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G186" s="3"/>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A187" s="2">
+        <v>46261</v>
+      </c>
+      <c r="B187" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C187" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D187" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E187" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F187" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G187" s="3"/>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A188" s="2">
+        <v>46262</v>
+      </c>
+      <c r="B188" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D188" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E188" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F188" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G188" s="3"/>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A189" s="2">
+        <v>46263</v>
+      </c>
+      <c r="B189" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C189" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D189" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E189" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F189" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G189" s="3"/>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A190" s="2">
+        <v>46264</v>
+      </c>
+      <c r="B190" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C190" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D190" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E190" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F190" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G190" s="3"/>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A191" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B191" s="21"/>
+      <c r="C191" s="3"/>
+      <c r="D191" s="3"/>
+      <c r="E191" s="3"/>
+      <c r="F191" s="3"/>
+      <c r="G191" s="3"/>
+    </row>
+    <row r="192" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A192" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="B192" s="20"/>
+      <c r="C192" s="20"/>
+      <c r="D192" s="20"/>
+      <c r="E192" s="20"/>
+      <c r="F192" s="20"/>
+      <c r="G192" s="20"/>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A193" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B193" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C193" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E193" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F193" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G193" s="3"/>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A194" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B194" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C194" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E194" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F194" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G194" s="3"/>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A195" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B195" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C195" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D195" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E195" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F195" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G195" s="3"/>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A196" s="2">
+        <v>46268</v>
+      </c>
+      <c r="B196" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C196" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E196" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F196" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G196" s="3"/>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A197" s="2">
+        <v>46269</v>
+      </c>
+      <c r="B197" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C197" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D197" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E197" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F197" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G197" s="3"/>
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A198" s="2">
+        <v>46270</v>
+      </c>
+      <c r="B198" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E198" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F198" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G198" s="3"/>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A199" s="2">
+        <v>46271</v>
+      </c>
+      <c r="B199" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C199" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D199" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E199" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F199" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G199" s="3"/>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A200" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B200" s="21"/>
+      <c r="C200" s="3"/>
+      <c r="D200" s="3"/>
+      <c r="E200" s="3"/>
+      <c r="F200" s="3"/>
+      <c r="G200" s="3"/>
+    </row>
+    <row r="201" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A201" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B201" s="20"/>
+      <c r="C201" s="20"/>
+      <c r="D201" s="20"/>
+      <c r="E201" s="20"/>
+      <c r="F201" s="20"/>
+      <c r="G201" s="20"/>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A202" s="2">
+        <v>46272</v>
+      </c>
+      <c r="B202" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D202" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E202" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F202" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G202" s="3"/>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A203" s="2">
+        <v>46273</v>
+      </c>
+      <c r="B203" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C203" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D203" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E203" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F203" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G203" s="3"/>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A204" s="2">
+        <v>46274</v>
+      </c>
+      <c r="B204" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C204" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D204" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E204" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F204" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G204" s="3"/>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A205" s="2">
+        <v>46275</v>
+      </c>
+      <c r="B205" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C205" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D205" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E205" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F205" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G205" s="3"/>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A206" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B206" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D206" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E206" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F206" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G206" s="3"/>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A207" s="2">
+        <v>46277</v>
+      </c>
+      <c r="B207" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C207" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D207" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E207" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F207" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G207" s="3"/>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A208" s="2">
+        <v>46278</v>
+      </c>
+      <c r="B208" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D208" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E208" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F208" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G208" s="3"/>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A209" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B209" s="21"/>
+      <c r="C209" s="3"/>
+      <c r="D209" s="3"/>
+      <c r="E209" s="3"/>
+      <c r="F209" s="3"/>
+      <c r="G209" s="3"/>
+    </row>
+    <row r="210" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A210" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B210" s="20"/>
+      <c r="C210" s="20"/>
+      <c r="D210" s="20"/>
+      <c r="E210" s="20"/>
+      <c r="F210" s="20"/>
+      <c r="G210" s="20"/>
+    </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A211" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B211" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C211" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D211" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E211" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F211" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G211" s="3"/>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A212" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B212" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E212" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F212" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G212" s="3"/>
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A213" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B213" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C213" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D213" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E213" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F213" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G213" s="3"/>
+    </row>
+    <row r="214" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A214" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B214" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D214" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E214" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F214" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G214" s="3"/>
+    </row>
+    <row r="215" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A215" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B215" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C215" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D215" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E215" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F215" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G215" s="3"/>
+    </row>
+    <row r="216" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A216" s="2">
+        <v>46284</v>
+      </c>
+      <c r="B216" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D216" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E216" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F216" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G216" s="3"/>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A217" s="2">
+        <v>46285</v>
+      </c>
+      <c r="B217" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C217" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D217" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E217" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F217" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G217" s="3"/>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A218" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B218" s="21"/>
+      <c r="C218" s="3"/>
+      <c r="D218" s="3"/>
+      <c r="E218" s="3"/>
+      <c r="F218" s="3"/>
+      <c r="G218" s="3"/>
+    </row>
+    <row r="219" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A219" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B219" s="20"/>
+      <c r="C219" s="20"/>
+      <c r="D219" s="20"/>
+      <c r="E219" s="20"/>
+      <c r="F219" s="20"/>
+      <c r="G219" s="20"/>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A220" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B220" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D220" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E220" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F220" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G220" s="3"/>
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A221" s="2">
+        <v>46287</v>
+      </c>
+      <c r="B221" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D221" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E221" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F221" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G221" s="3"/>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A222" s="2">
+        <v>46288</v>
+      </c>
+      <c r="B222" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D222" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E222" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F222" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G222" s="3"/>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A223" s="2">
+        <v>46289</v>
+      </c>
+      <c r="B223" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D223" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E223" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F223" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G223" s="3"/>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A224" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B224" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C224" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D224" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E224" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F224" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G224" s="3"/>
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A225" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B225" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D225" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E225" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F225" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G225" s="3"/>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A226" s="2">
+        <v>46292</v>
+      </c>
+      <c r="B226" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D226" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E226" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F226" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G226" s="3"/>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A227" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B227" s="21"/>
+      <c r="C227" s="3"/>
+      <c r="D227" s="3"/>
+      <c r="E227" s="3"/>
+      <c r="F227" s="3"/>
+      <c r="G227" s="3"/>
+    </row>
+    <row r="228" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+      <c r="A228" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B228" s="20"/>
+      <c r="C228" s="20"/>
+      <c r="D228" s="20"/>
+      <c r="E228" s="20"/>
+      <c r="F228" s="20"/>
+      <c r="G228" s="20"/>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A229" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B229" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D229" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E229" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F229" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G229" s="3"/>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A230" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B230" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D230" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E230" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F230" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G230" s="3"/>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A231" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B231" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D231" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E231" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F231" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G231" s="3"/>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A232" s="2">
+        <v>46296</v>
+      </c>
+      <c r="B232" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D232" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E232" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F232" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G232" s="3"/>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A233" s="2">
+        <v>46297</v>
+      </c>
+      <c r="B233" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D233" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E233" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F233" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G233" s="3"/>
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A234" s="2">
+        <v>46298</v>
+      </c>
+      <c r="B234" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E234" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F234" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G234" s="3"/>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A235" s="2">
+        <v>46299</v>
+      </c>
+      <c r="B235" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D235" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E235" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F235" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G235" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="39">
+    <mergeCell ref="A219:G219"/>
+    <mergeCell ref="A228:G228"/>
+    <mergeCell ref="A174:G174"/>
+    <mergeCell ref="A183:G183"/>
+    <mergeCell ref="A192:G192"/>
+    <mergeCell ref="A201:G201"/>
+    <mergeCell ref="A210:G210"/>
+    <mergeCell ref="A129:G129"/>
+    <mergeCell ref="A138:G138"/>
+    <mergeCell ref="A147:G147"/>
+    <mergeCell ref="A156:G156"/>
+    <mergeCell ref="A165:G165"/>
+    <mergeCell ref="A3:G4"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A54:G54"/>
     <mergeCell ref="D55:D56"/>
     <mergeCell ref="E55:E56"/>
     <mergeCell ref="F55:F56"/>
@@ -3462,19 +5498,6 @@
     <mergeCell ref="A55:A56"/>
     <mergeCell ref="B55:B56"/>
     <mergeCell ref="C55:C56"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="A3:G4"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>